<commit_message>
HbA1c: added label to target codes
</commit_message>
<xml_diff>
--- a/codelists/HbA1c_raw.xlsx
+++ b/codelists/HbA1c_raw.xlsx
@@ -410,7 +410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.48" customWidth="1" min="1" max="1"/>
@@ -422,12 +422,13 @@
     <col width="140.76" customWidth="1" min="7" max="7"/>
     <col width="6.44" customWidth="1" min="8" max="8"/>
     <col width="20.24" customWidth="1" min="9" max="9"/>
-    <col width="11.96" customWidth="1" min="10" max="10"/>
-    <col width="17.48" customWidth="1" min="11" max="11"/>
-    <col width="16.56" customWidth="1" min="12" max="12"/>
-    <col width="11.96" customWidth="1" min="13" max="13"/>
-    <col width="16.56" customWidth="1" min="14" max="14"/>
-    <col width="15.64" customWidth="1" min="15" max="15"/>
+    <col width="7.36" customWidth="1" min="10" max="10"/>
+    <col width="11.96" customWidth="1" min="11" max="11"/>
+    <col width="17.48" customWidth="1" min="12" max="12"/>
+    <col width="16.56" customWidth="1" min="13" max="13"/>
+    <col width="11.96" customWidth="1" min="14" max="14"/>
+    <col width="16.56" customWidth="1" min="15" max="15"/>
+    <col width="15.64" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,30 +479,35 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>hba1c_tests</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>hba1c_tests_value</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>refset_dccthba1c</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>hba1c_value</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>refset_ifcchbamd</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>refset_ifcchbam</t>
         </is>
@@ -547,20 +553,21 @@
       <c r="I2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="1" t="n">
-        <v>1</v>
-      </c>
+      <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="1" t="n"/>
-      <c r="M2" s="1" t="n">
-        <v>1</v>
-      </c>
+      <c r="L2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="1" t="n"/>
       <c r="N2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="O2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -604,14 +611,15 @@
       <c r="I3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L3" s="1" t="n"/>
       <c r="M3" s="1" t="n"/>
       <c r="N3" s="1" t="n"/>
       <c r="O3" s="1" t="n"/>
+      <c r="P3" s="1" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -653,14 +661,15 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L4" s="1" t="n"/>
       <c r="M4" s="1" t="n"/>
       <c r="N4" s="1" t="n"/>
       <c r="O4" s="1" t="n"/>
+      <c r="P4" s="1" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -698,14 +707,15 @@
       <c r="I5" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="1" t="n"/>
+      <c r="J5" s="1" t="n"/>
+      <c r="K5" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L5" s="1" t="n"/>
       <c r="M5" s="1" t="n"/>
       <c r="N5" s="1" t="n"/>
       <c r="O5" s="1" t="n"/>
+      <c r="P5" s="1" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -743,14 +753,15 @@
       <c r="I6" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L6" s="1" t="n"/>
       <c r="M6" s="1" t="n"/>
       <c r="N6" s="1" t="n"/>
       <c r="O6" s="1" t="n"/>
+      <c r="P6" s="1" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -788,14 +799,15 @@
       <c r="I7" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="1" t="n"/>
+      <c r="J7" s="1" t="n"/>
+      <c r="K7" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L7" s="1" t="n"/>
       <c r="M7" s="1" t="n"/>
       <c r="N7" s="1" t="n"/>
       <c r="O7" s="1" t="n"/>
+      <c r="P7" s="1" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -833,14 +845,15 @@
       <c r="I8" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L8" s="1" t="n"/>
       <c r="M8" s="1" t="n"/>
       <c r="N8" s="1" t="n"/>
       <c r="O8" s="1" t="n"/>
+      <c r="P8" s="1" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -878,14 +891,15 @@
       <c r="I9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1" t="n"/>
+      <c r="J9" s="1" t="n"/>
+      <c r="K9" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
       <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -923,14 +937,15 @@
       <c r="I10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1" t="n"/>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L10" s="1" t="n"/>
       <c r="M10" s="1" t="n"/>
       <c r="N10" s="1" t="n"/>
       <c r="O10" s="1" t="n"/>
+      <c r="P10" s="1" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -968,14 +983,15 @@
       <c r="I11" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+      <c r="K11" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L11" s="1" t="n"/>
       <c r="M11" s="1" t="n"/>
       <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="n"/>
+      <c r="P11" s="1" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1013,14 +1029,15 @@
       <c r="I12" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="1" t="n"/>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="L12" s="1" t="n"/>
       <c r="M12" s="1" t="n"/>
       <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="n"/>
+      <c r="P12" s="1" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1064,14 +1081,15 @@
       </c>
       <c r="J13" s="1" t="n"/>
       <c r="K13" s="1" t="n"/>
-      <c r="L13" s="1" t="n">
-        <v>1</v>
-      </c>
+      <c r="L13" s="1" t="n"/>
       <c r="M13" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="N13" s="1" t="n"/>
+      <c r="N13" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="O13" s="1" t="n"/>
+      <c r="P13" s="1" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1112,11 +1130,12 @@
       <c r="J14" s="1" t="n"/>
       <c r="K14" s="1" t="n"/>
       <c r="L14" s="1" t="n"/>
-      <c r="M14" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="1" t="n"/>
-      <c r="O14" s="1" t="n">
+      <c r="M14" s="1" t="n"/>
+      <c r="N14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="1" t="n"/>
+      <c r="P14" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1159,11 +1178,12 @@
       <c r="J15" s="1" t="n"/>
       <c r="K15" s="1" t="n"/>
       <c r="L15" s="1" t="n"/>
-      <c r="M15" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="1" t="n"/>
-      <c r="O15" s="1" t="n">
+      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="n"/>
+      <c r="P15" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1206,11 +1226,12 @@
       <c r="J16" s="1" t="n"/>
       <c r="K16" s="1" t="n"/>
       <c r="L16" s="1" t="n"/>
-      <c r="M16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="1" t="n"/>
+      <c r="M16" s="1" t="n"/>
+      <c r="N16" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="O16" s="1" t="n"/>
+      <c r="P16" s="1" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1251,11 +1272,12 @@
       <c r="J17" s="1" t="n"/>
       <c r="K17" s="1" t="n"/>
       <c r="L17" s="1" t="n"/>
-      <c r="M17" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N17" s="1" t="n"/>
+      <c r="M17" s="1" t="n"/>
+      <c r="N17" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="O17" s="1" t="n"/>
+      <c r="P17" s="1" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1296,11 +1318,12 @@
       <c r="J18" s="1" t="n"/>
       <c r="K18" s="1" t="n"/>
       <c r="L18" s="1" t="n"/>
-      <c r="M18" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="1" t="n"/>
+      <c r="M18" s="1" t="n"/>
+      <c r="N18" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="O18" s="1" t="n"/>
+      <c r="P18" s="1" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1348,6 +1371,7 @@
       <c r="M19" s="1" t="n"/>
       <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="n"/>
+      <c r="P19" s="1" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1395,6 +1419,7 @@
       <c r="M20" s="1" t="n"/>
       <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
+      <c r="P20" s="1" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1442,6 +1467,7 @@
       <c r="M21" s="1" t="n"/>
       <c r="N21" s="1" t="n"/>
       <c r="O21" s="1" t="n"/>
+      <c r="P21" s="1" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1483,12 +1509,15 @@
       <c r="I22" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="1" t="n"/>
+      <c r="J22" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K22" s="1" t="n"/>
       <c r="L22" s="1" t="n"/>
       <c r="M22" s="1" t="n"/>
       <c r="N22" s="1" t="n"/>
       <c r="O22" s="1" t="n"/>
+      <c r="P22" s="1" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1536,6 +1565,7 @@
       <c r="M23" s="1" t="n"/>
       <c r="N23" s="1" t="n"/>
       <c r="O23" s="1" t="n"/>
+      <c r="P23" s="1" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1583,6 +1613,7 @@
       <c r="M24" s="1" t="n"/>
       <c r="N24" s="1" t="n"/>
       <c r="O24" s="1" t="n"/>
+      <c r="P24" s="1" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1630,6 +1661,7 @@
       <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
       <c r="O25" s="1" t="n"/>
+      <c r="P25" s="1" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1677,6 +1709,7 @@
       <c r="M26" s="1" t="n"/>
       <c r="N26" s="1" t="n"/>
       <c r="O26" s="1" t="n"/>
+      <c r="P26" s="1" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1718,12 +1751,15 @@
       <c r="I27" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="1" t="n"/>
+      <c r="J27" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K27" s="1" t="n"/>
       <c r="L27" s="1" t="n"/>
       <c r="M27" s="1" t="n"/>
       <c r="N27" s="1" t="n"/>
       <c r="O27" s="1" t="n"/>
+      <c r="P27" s="1" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1771,6 +1807,7 @@
       <c r="M28" s="1" t="n"/>
       <c r="N28" s="1" t="n"/>
       <c r="O28" s="1" t="n"/>
+      <c r="P28" s="1" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1808,12 +1845,15 @@
       <c r="I29" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="1" t="n"/>
+      <c r="J29" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" s="1" t="n"/>
       <c r="L29" s="1" t="n"/>
       <c r="M29" s="1" t="n"/>
       <c r="N29" s="1" t="n"/>
       <c r="O29" s="1" t="n"/>
+      <c r="P29" s="1" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1861,6 +1901,7 @@
       <c r="M30" s="1" t="n"/>
       <c r="N30" s="1" t="n"/>
       <c r="O30" s="1" t="n"/>
+      <c r="P30" s="1" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1908,6 +1949,7 @@
       <c r="M31" s="1" t="n"/>
       <c r="N31" s="1" t="n"/>
       <c r="O31" s="1" t="n"/>
+      <c r="P31" s="1" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1951,6 +1993,7 @@
       <c r="M32" s="1" t="n"/>
       <c r="N32" s="1" t="n"/>
       <c r="O32" s="1" t="n"/>
+      <c r="P32" s="1" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1998,6 +2041,7 @@
       <c r="M33" s="1" t="n"/>
       <c r="N33" s="1" t="n"/>
       <c r="O33" s="1" t="n"/>
+      <c r="P33" s="1" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2045,6 +2089,7 @@
       <c r="M34" s="1" t="n"/>
       <c r="N34" s="1" t="n"/>
       <c r="O34" s="1" t="n"/>
+      <c r="P34" s="1" t="n"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2092,6 +2137,7 @@
       <c r="M35" s="1" t="n"/>
       <c r="N35" s="1" t="n"/>
       <c r="O35" s="1" t="n"/>
+      <c r="P35" s="1" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2129,12 +2175,15 @@
       <c r="I36" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J36" s="1" t="n"/>
+      <c r="J36" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K36" s="1" t="n"/>
       <c r="L36" s="1" t="n"/>
       <c r="M36" s="1" t="n"/>
       <c r="N36" s="1" t="n"/>
       <c r="O36" s="1" t="n"/>
+      <c r="P36" s="1" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2178,6 +2227,7 @@
       <c r="M37" s="1" t="n"/>
       <c r="N37" s="1" t="n"/>
       <c r="O37" s="1" t="n"/>
+      <c r="P37" s="1" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2221,6 +2271,7 @@
       <c r="M38" s="1" t="n"/>
       <c r="N38" s="1" t="n"/>
       <c r="O38" s="1" t="n"/>
+      <c r="P38" s="1" t="n"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2258,12 +2309,15 @@
       <c r="I39" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J39" s="1" t="n"/>
+      <c r="J39" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K39" s="1" t="n"/>
       <c r="L39" s="1" t="n"/>
       <c r="M39" s="1" t="n"/>
       <c r="N39" s="1" t="n"/>
       <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2307,6 +2361,7 @@
       <c r="M40" s="1" t="n"/>
       <c r="N40" s="1" t="n"/>
       <c r="O40" s="1" t="n"/>
+      <c r="P40" s="1" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2350,6 +2405,7 @@
       <c r="M41" s="1" t="n"/>
       <c r="N41" s="1" t="n"/>
       <c r="O41" s="1" t="n"/>
+      <c r="P41" s="1" t="n"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2393,6 +2449,7 @@
       <c r="M42" s="1" t="n"/>
       <c r="N42" s="1" t="n"/>
       <c r="O42" s="1" t="n"/>
+      <c r="P42" s="1" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2436,6 +2493,7 @@
       <c r="M43" s="1" t="n"/>
       <c r="N43" s="1" t="n"/>
       <c r="O43" s="1" t="n"/>
+      <c r="P43" s="1" t="n"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2479,6 +2537,7 @@
       <c r="M44" s="1" t="n"/>
       <c r="N44" s="1" t="n"/>
       <c r="O44" s="1" t="n"/>
+      <c r="P44" s="1" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2516,12 +2575,15 @@
       <c r="I45" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J45" s="1" t="n"/>
+      <c r="J45" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K45" s="1" t="n"/>
       <c r="L45" s="1" t="n"/>
       <c r="M45" s="1" t="n"/>
       <c r="N45" s="1" t="n"/>
       <c r="O45" s="1" t="n"/>
+      <c r="P45" s="1" t="n"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2565,6 +2627,7 @@
       <c r="M46" s="1" t="n"/>
       <c r="N46" s="1" t="n"/>
       <c r="O46" s="1" t="n"/>
+      <c r="P46" s="1" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2602,12 +2665,15 @@
       <c r="I47" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J47" s="1" t="n"/>
+      <c r="J47" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K47" s="1" t="n"/>
       <c r="L47" s="1" t="n"/>
       <c r="M47" s="1" t="n"/>
       <c r="N47" s="1" t="n"/>
       <c r="O47" s="1" t="n"/>
+      <c r="P47" s="1" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2645,12 +2711,15 @@
       <c r="I48" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J48" s="1" t="n"/>
+      <c r="J48" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K48" s="1" t="n"/>
       <c r="L48" s="1" t="n"/>
       <c r="M48" s="1" t="n"/>
       <c r="N48" s="1" t="n"/>
       <c r="O48" s="1" t="n"/>
+      <c r="P48" s="1" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2694,6 +2763,7 @@
       <c r="M49" s="1" t="n"/>
       <c r="N49" s="1" t="n"/>
       <c r="O49" s="1" t="n"/>
+      <c r="P49" s="1" t="n"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2731,12 +2801,15 @@
       <c r="I50" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J50" s="1" t="n"/>
+      <c r="J50" s="1" t="n">
+        <v>1</v>
+      </c>
       <c r="K50" s="1" t="n"/>
       <c r="L50" s="1" t="n"/>
       <c r="M50" s="1" t="n"/>
       <c r="N50" s="1" t="n"/>
       <c r="O50" s="1" t="n"/>
+      <c r="P50" s="1" t="n"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2780,6 +2853,7 @@
       <c r="M51" s="1" t="n"/>
       <c r="N51" s="1" t="n"/>
       <c r="O51" s="1" t="n"/>
+      <c r="P51" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>